<commit_message>
add image link to excel
</commit_message>
<xml_diff>
--- a/data/bs1_product.xlsx
+++ b/data/bs1_product.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="23760"/>
+    <workbookView windowHeight="17200"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>No.</t>
   </si>
@@ -115,16 +115,27 @@
     <t>language</t>
   </si>
   <si>
+    <t>pic_path</t>
+  </si>
+  <si>
     <t>https://s.shopee.co.th/8ARASSGaRk</t>
   </si>
   <si>
     <t>th</t>
   </si>
   <si>
+    <t>https://down-th.img.susercontent.com/file/th-11134207-81zto-mjxqwdgg5fyc33@resize_w900_nl.webp
+https://down-th.img.susercontent.com/file/th-11134207-7r98w-lx7t8vw9kybza1</t>
+  </si>
+  <si>
     <t>https://s.shopee.co.th/15SjUy0Xa</t>
   </si>
   <si>
     <t>https://s.shopee.co.th/7poK3uNwJv</t>
+  </si>
+  <si>
+    <t>https://down-th.img.susercontent.com/file/th-11134207-7ra0q-mbtfcuxlt6xf5f@resize_w900_nl.webp
+https://down-th.img.susercontent.com/file/th-11134207-7r992-lx11ypfajqofc7</t>
   </si>
   <si>
     <t>https://s.shopee.co.th/9UwY33B2Or</t>
@@ -164,7 +175,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,13 +212,6 @@
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -674,19 +678,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -695,7 +699,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -704,118 +711,115 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -834,7 +838,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1181,17 +1185,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="5" outlineLevelCol="4"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="68" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="55.984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1207,87 +1212,101 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" ht="17" spans="1:5">
+    <row r="2" ht="68" spans="1:6">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3" ht="17" spans="1:5">
+    <row r="3" ht="17" spans="1:6">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F3" s="3"/>
     </row>
-    <row r="4" ht="17" spans="1:5">
+    <row r="4" ht="68" spans="1:6">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3"/>
-      <c r="C4" s="4" t="s">
-        <v>8</v>
+      <c r="C4" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" ht="17" spans="1:5">
+    <row r="5" ht="17" spans="1:6">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
-    <row r="6" ht="17" spans="1:5">
+    <row r="6" ht="17" spans="1:6">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F6" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D3 D4:D6 D7:D977">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D977">
       <formula1>"shopee,tiktok,facebook,instagram"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E3 E4:E6 E7:E977">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E977">
       <formula1>"th,en"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId3" display="https://s.shopee.co.th/8ARASSGaRk"/>
-    <hyperlink ref="C3" r:id="rId4" display="https://s.shopee.co.th/15SjUy0Xa"/>
+    <hyperlink ref="C2" r:id="rId3" display="https://s.shopee.co.th/8ARASSGaRk" tooltip="https://s.shopee.co.th/8ARASSGaRk"/>
+    <hyperlink ref="C3" r:id="rId4" display="https://s.shopee.co.th/15SjUy0Xa" tooltip="https://s.shopee.co.th/15SjUy0Xa"/>
     <hyperlink ref="C4" r:id="rId5" display="https://s.shopee.co.th/7poK3uNwJv"/>
     <hyperlink ref="C5" r:id="rId6" display="https://s.shopee.co.th/9UwY33B2Or"/>
     <hyperlink ref="C6" r:id="rId7" display="https://s.shopee.co.th/9fFyFMAP3u"/>
+    <hyperlink ref="F2" r:id="rId8" display="https://down-th.img.susercontent.com/file/th-11134207-81zto-mjxqwdgg5fyc33@resize_w900_nl.webp&#10;https://down-th.img.susercontent.com/file/th-11134207-7r98w-lx7t8vw9kybza1" tooltip="https://down-th.img.susercontent.com/file/th-11134207-81zto-mjxqwdgg5fyc33@resize_w900_nl.webp"/>
+    <hyperlink ref="F4" r:id="rId9" display="https://down-th.img.susercontent.com/file/th-11134207-7ra0q-mbtfcuxlt6xf5f@resize_w900_nl.webp&#10;https://down-th.img.susercontent.com/file/th-11134207-7r992-lx11ypfajqofc7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1306,37 +1325,37 @@
   <sheetData>
     <row r="1" ht="20.4" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>